<commit_message>
Agregar hoja de verificacion de irregularidad torsional al Excel base (insercion quirurgica, conserva imagenes y graficos)
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Proyecto diseño (1).xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Proyecto diseño (1).xlsx
@@ -26,6 +26,7 @@
     <sheet name="FHE " sheetId="23" r:id="rId11"/>
     <sheet name="FHE  (2)" sheetId="27" r:id="rId12"/>
     <sheet name="Derivas" sheetId="25" r:id="rId13"/>
+    <sheet name="Irreg. Torsional" sheetId="28" r:id="rId28"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId14"/>
@@ -1184,7 +1185,7 @@
     <numFmt numFmtId="167" formatCode="0.00000000000000"/>
     <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1387,6 +1388,18 @@
       <color theme="1"/>
       <name val="Ancizar Serif"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F4E79"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="13">
@@ -2131,7 +2144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="396">
+  <cellXfs count="398">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3200,6 +3213,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13337,6 +13354,418 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VERIFICACIÓN DE IRREGULARIDAD TORSIONAL EN PLANTA (NSR-10 A.3.6.7 — Tipo 1aP/1bP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criterio:  razón = δmax / δprom ,  con δprom = (δmax + δmin)/2 entre los dos bordes del diafragma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular si razón ≤ 1.20  |  Torsional 1aP (φp=0.9) si 1.20 &lt; razón ≤ 1.40  |  Extrema 1bP (φp=0.8) si &gt; 1.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desplazamientos de SAP2000 (Joint Displacements), TODOS los nudos de cada diafragma. U1 para Fx, U2 para Fy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SISMO EN X (Fx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso Z (m)</t>
+        </is>
+      </c>
+      <c r="B8" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N° nudos</t>
+        </is>
+      </c>
+      <c r="C8" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">δmax (mm)</t>
+        </is>
+      </c>
+      <c r="D8" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">δmin (mm)</t>
+        </is>
+      </c>
+      <c r="E8" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">δprom (mm)</t>
+        </is>
+      </c>
+      <c r="F8" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">razón</t>
+        </is>
+      </c>
+      <c r="G8" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="B9" s="0">
+        <v>183</v>
+      </c>
+      <c r="C9" s="0">
+        <v>24.099</v>
+      </c>
+      <c r="D9" s="0">
+        <v>22.986</v>
+      </c>
+      <c r="E9" s="0">
+        <v>23.543</v>
+      </c>
+      <c r="F9" s="0">
+        <v>1.024</v>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>6.5</v>
+      </c>
+      <c r="B10" s="0">
+        <v>183</v>
+      </c>
+      <c r="C10" s="0">
+        <v>54.676</v>
+      </c>
+      <c r="D10" s="0">
+        <v>52.244</v>
+      </c>
+      <c r="E10" s="0">
+        <v>53.46</v>
+      </c>
+      <c r="F10" s="0">
+        <v>1.023</v>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>9.5</v>
+      </c>
+      <c r="B11" s="0">
+        <v>183</v>
+      </c>
+      <c r="C11" s="0">
+        <v>81.98</v>
+      </c>
+      <c r="D11" s="0">
+        <v>78.404</v>
+      </c>
+      <c r="E11" s="0">
+        <v>80.192</v>
+      </c>
+      <c r="F11" s="0">
+        <v>1.022</v>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>12.5</v>
+      </c>
+      <c r="B12" s="0">
+        <v>183</v>
+      </c>
+      <c r="C12" s="0">
+        <v>101.698</v>
+      </c>
+      <c r="D12" s="0">
+        <v>97.317</v>
+      </c>
+      <c r="E12" s="0">
+        <v>99.507</v>
+      </c>
+      <c r="F12" s="0">
+        <v>1.022</v>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>15.5</v>
+      </c>
+      <c r="B13" s="0">
+        <v>183</v>
+      </c>
+      <c r="C13" s="0">
+        <v>112.878</v>
+      </c>
+      <c r="D13" s="0">
+        <v>108.069</v>
+      </c>
+      <c r="E13" s="0">
+        <v>110.474</v>
+      </c>
+      <c r="F13" s="0">
+        <v>1.022</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SISMO EN Y (Fy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso Z (m)</t>
+        </is>
+      </c>
+      <c r="B16" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N° nudos</t>
+        </is>
+      </c>
+      <c r="C16" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">δmax (mm)</t>
+        </is>
+      </c>
+      <c r="D16" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">δmin (mm)</t>
+        </is>
+      </c>
+      <c r="E16" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">δprom (mm)</t>
+        </is>
+      </c>
+      <c r="F16" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">razón</t>
+        </is>
+      </c>
+      <c r="G16" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="B17" s="0">
+        <v>183</v>
+      </c>
+      <c r="C17" s="0">
+        <v>20.97</v>
+      </c>
+      <c r="D17" s="0">
+        <v>20.419</v>
+      </c>
+      <c r="E17" s="0">
+        <v>20.694</v>
+      </c>
+      <c r="F17" s="0">
+        <v>1.013</v>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>6.5</v>
+      </c>
+      <c r="B18" s="0">
+        <v>183</v>
+      </c>
+      <c r="C18" s="0">
+        <v>43.378</v>
+      </c>
+      <c r="D18" s="0">
+        <v>42.175</v>
+      </c>
+      <c r="E18" s="0">
+        <v>42.776</v>
+      </c>
+      <c r="F18" s="0">
+        <v>1.014</v>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>9.5</v>
+      </c>
+      <c r="B19" s="0">
+        <v>183</v>
+      </c>
+      <c r="C19" s="0">
+        <v>62.5</v>
+      </c>
+      <c r="D19" s="0">
+        <v>60.732</v>
+      </c>
+      <c r="E19" s="0">
+        <v>61.616</v>
+      </c>
+      <c r="F19" s="0">
+        <v>1.014</v>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>12.5</v>
+      </c>
+      <c r="B20" s="0">
+        <v>183</v>
+      </c>
+      <c r="C20" s="0">
+        <v>75.919</v>
+      </c>
+      <c r="D20" s="0">
+        <v>73.753</v>
+      </c>
+      <c r="E20" s="0">
+        <v>74.836</v>
+      </c>
+      <c r="F20" s="0">
+        <v>1.014</v>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>15.5</v>
+      </c>
+      <c r="B21" s="0">
+        <v>183</v>
+      </c>
+      <c r="C21" s="0">
+        <v>82.785</v>
+      </c>
+      <c r="D21" s="0">
+        <v>80.409</v>
+      </c>
+      <c r="E21" s="0">
+        <v>81.597</v>
+      </c>
+      <c r="F21" s="0">
+        <v>1.015</v>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regular</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAZÓN MÁXIMA = 1.024  &lt;  1.20   →   NO HAY IRREGULARIDAD TORSIONAL   →   φp = 1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con planta, altura y redundancia regulares:  R = R0·φa·φp·φr = 5·1·1·1 = 5.0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C4147E5-6826-45DD-A297-30816CF08B5A}">
   <dimension ref="A14:R93"/>

</xml_diff>

<commit_message>
Planos de despiece actualizados (VC-1..9, VR-1..11, viguetas, riostras cimentacion) + hoja Viguetas C.8.3.3 en Excel base
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Proyecto diseño (1).xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Proyecto diseño (1).xlsx
@@ -27,6 +27,7 @@
     <sheet name="FHE  (2)" sheetId="27" r:id="rId12"/>
     <sheet name="Derivas" sheetId="25" r:id="rId13"/>
     <sheet name="Irreg. Torsional" sheetId="28" r:id="rId28"/>
+    <sheet name="Viguetas C.8.3.3" sheetId="29" r:id="rId29"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId14"/>
@@ -13766,6 +13767,299 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DISEÑO DE VIGUETAS — Momentos por coeficientes NSR-10 C.8.3.3 (según tipo de apoyo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Losa aligerada en una dirección. Nervio 0.15 x 0.34 m + loseta 0.06 m. Sep. 0.80 m. d=304 mm. As_min=152 mm². 2 Nº4 = 258 mm².</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Código de apoyo</t>
+        </is>
+      </c>
+      <c r="B5" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condición</t>
+        </is>
+      </c>
+      <c r="C5" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M+ (positivo)</t>
+        </is>
+      </c>
+      <c r="D5" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M- (negativo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1EC</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vano extremo (un extremo continuo)</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wu·ln²/14</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1er apoyo interior: wu·ln²/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2EC</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vano interior (dos extremos continuos)</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wu·ln²/16</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">en apoyos: wu·ln²/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(ext.)</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apoyo exterior monolítico con viga</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wu·ln²/24</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voladizo</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wu·L²/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verificación de los casos gobernantes (wu entrepiso=9.06 kN/m; cubierta terraza=10.6 kN/m):</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caso gobernante</t>
+        </is>
+      </c>
+      <c r="B12" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ln (m)</t>
+        </is>
+      </c>
+      <c r="C12" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wu (kN/m)</t>
+        </is>
+      </c>
+      <c r="D12" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M- (kN·m)</t>
+        </is>
+      </c>
+      <c r="E12" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M+ (kN·m)</t>
+        </is>
+      </c>
+      <c r="F12" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As req (mm²)</t>
+        </is>
+      </c>
+      <c r="G12" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Refuerzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrepiso, vano extremo 1EC</t>
+        </is>
+      </c>
+      <c r="B13" s="0">
+        <v>4.75</v>
+      </c>
+      <c r="C13" s="0">
+        <v>9.06</v>
+      </c>
+      <c r="D13" s="0">
+        <v>20.4</v>
+      </c>
+      <c r="E13" s="0">
+        <v>14.6</v>
+      </c>
+      <c r="F13" s="0">
+        <v>185</v>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cubierta, vano 1EC (terraza L=5)</t>
+        </is>
+      </c>
+      <c r="B14" s="0">
+        <v>4.75</v>
+      </c>
+      <c r="C14" s="0">
+        <v>10.6</v>
+      </c>
+      <c r="D14" s="0">
+        <v>23.9</v>
+      </c>
+      <c r="E14" s="0">
+        <v>17.1</v>
+      </c>
+      <c r="F14" s="0">
+        <v>217</v>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voladizo V 1.5 m</t>
+        </is>
+      </c>
+      <c r="B15" s="0">
+        <v>1.27</v>
+      </c>
+      <c r="C15" s="0">
+        <v>9.06</v>
+      </c>
+      <c r="D15" s="0">
+        <v>10.2</v>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F15" s="0">
+        <v>152</v>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCLUSIÓN: aun con el coeficiente más exigente de cada apoyo, As req (máx 217 mm²) &lt; 2 Nº4 (258) → gobierna acero mínimo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cortante: Vu,máx = 29.3 kN &lt; φ·(1.1·Vc) → no se requieren estribos (C.8.3.3 permite incrementar Vc 10% en viguetas).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C4147E5-6826-45DD-A297-30816CF08B5A}">
   <dimension ref="A14:R93"/>

</xml_diff>